<commit_message>
expt 2 results corrected
</commit_message>
<xml_diff>
--- a/Results/Study 2/AlexNet (pretrained)/Confusion Matrices.xlsx
+++ b/Results/Study 2/AlexNet (pretrained)/Confusion Matrices.xlsx
@@ -400,10 +400,10 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>485</v>
+        <v>546</v>
       </c>
       <c r="C2">
-        <v>155</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -411,10 +411,10 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>189</v>
+        <v>516</v>
       </c>
       <c r="C3">
-        <v>451</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -440,10 +440,10 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -451,10 +451,10 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>68</v>
+        <v>128</v>
       </c>
       <c r="C3">
-        <v>92</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>